<commit_message>
chore: run 2026-03-31 10:13 — histórico, dashboard e Excel atualizados
</commit_message>
<xml_diff>
--- a/logs/Consolidado_31_03_2026.xlsx
+++ b/logs/Consolidado_31_03_2026.xlsx
@@ -641,7 +641,7 @@
         <v>8</v>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
@@ -663,7 +663,7 @@
         <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
@@ -676,7 +676,7 @@
         <v>77</v>
       </c>
       <c r="C4" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D4" t="n">
         <v>1</v>
@@ -8358,13 +8358,7 @@
           <t>Ducray</t>
         </is>
       </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>Emulsão Crosta Láctea Kelual
-Emulsão Crosta Láctea Calmante Pele do Bebé
-50 ml</t>
-        </is>
-      </c>
+      <c r="C24" s="3" t="inlineStr"/>
       <c r="D24" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/emulsao-crosta-lactea-kelual-3066114.html</t>
@@ -8376,14 +8370,10 @@
           <t>In Stock</t>
         </is>
       </c>
-      <c r="G24" s="3" t="inlineStr">
-        <is>
-          <t>3066114</t>
-        </is>
-      </c>
+      <c r="G24" s="3" t="inlineStr"/>
       <c r="H24" s="3" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>Sem desconto</t>
         </is>
       </c>
     </row>
@@ -8398,13 +8388,7 @@
           <t>Ducray</t>
         </is>
       </c>
-      <c r="C25" s="5" t="inlineStr">
-        <is>
-          <t>Extra Doux Shampooing Dermo-Protecteur
-Champô Ultra Suave para Uso Familiar
-100 ml</t>
-        </is>
-      </c>
+      <c r="C25" s="5" t="inlineStr"/>
       <c r="D25" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/extra-doux-shampooing-dermo-protecteur-5797814.html</t>
@@ -8416,14 +8400,10 @@
           <t>In Stock</t>
         </is>
       </c>
-      <c r="G25" s="5" t="inlineStr">
-        <is>
-          <t>5797814</t>
-        </is>
-      </c>
+      <c r="G25" s="5" t="inlineStr"/>
       <c r="H25" s="5" t="inlineStr">
         <is>
-          <t>20%</t>
+          <t>Sem desconto</t>
         </is>
       </c>
     </row>
@@ -11369,40 +11349,40 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="5" t="inlineStr">
-        <is>
-          <t>31/03/2026</t>
-        </is>
-      </c>
-      <c r="B26" s="5" t="inlineStr">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>31/03/2026</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="C26" s="5" t="inlineStr">
+      <c r="C26" s="7" t="inlineStr">
         <is>
           <t>Cupuaçu BIO Gel Duche Nutritivo Hibiscus
 Gel Duche Hidratante Flor de Hibísco
 200 ml</t>
         </is>
       </c>
-      <c r="D26" s="5" t="inlineStr">
+      <c r="D26" s="7" t="inlineStr">
         <is>
           <t>https://wells.pt/cupuacu-bio-gel-duche-nutritivo-hibiscus-6515228.html</t>
         </is>
       </c>
-      <c r="E26" s="5" t="inlineStr"/>
-      <c r="F26" s="6" t="inlineStr">
-        <is>
-          <t>In Stock</t>
-        </is>
-      </c>
-      <c r="G26" s="5" t="inlineStr">
+      <c r="E26" s="7" t="inlineStr"/>
+      <c r="F26" s="8" t="inlineStr">
+        <is>
+          <t>Out of Stock</t>
+        </is>
+      </c>
+      <c r="G26" s="7" t="inlineStr">
         <is>
           <t>6515228</t>
         </is>
       </c>
-      <c r="H26" s="5" t="inlineStr">
+      <c r="H26" s="7" t="inlineStr">
         <is>
           <t>25%</t>
         </is>

</xml_diff>